<commit_message>
Sync UAT workbook values from dev
</commit_message>
<xml_diff>
--- a/Dev_Test_Ops/KPI_TEST_DASHBOARD - UAT.xlsx
+++ b/Dev_Test_Ops/KPI_TEST_DASHBOARD - UAT.xlsx
@@ -997,11 +997,11 @@
         <v>12</v>
       </c>
       <c r="G19" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H19" s="3">
         <f t="shared" ref="H19" si="2">IF(AND(ISNUMBER(G19),ISNUMBER(E19)),IF(E19&lt;&gt;0,(G19/E19)*100,""),"")</f>
-        <v>91.42857142857143</v>
+        <v>92.85714285714286</v>
       </c>
       <c r="I19" t="str">
         <f t="shared" ref="I19" si="3">IF(G19="","",IF(F19="&gt;=",IF(G19&gt;=E19,"Met","Not Met"),IF(F19="&lt;=",IF(G19&lt;=E19,"Met","Not Met"),IF(F19="=",IF(G19=E19,"Met","Not Met"),""))))</f>
@@ -1025,11 +1025,11 @@
         <v>27</v>
       </c>
       <c r="G20" s="2">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H20" s="3">
         <f t="shared" ref="H20" si="4">IF(AND(ISNUMBER(G20),ISNUMBER(E20)),IF(E20&lt;&gt;0,(G20/E20)*100,""),"")</f>
-        <v>88.75</v>
+        <v>86.25</v>
       </c>
       <c r="I20" t="str">
         <f t="shared" ref="I20" si="5">IF(G20="","",IF(F20="&gt;=",IF(G20&gt;=E20,"Met","Not Met"),IF(F20="&lt;=",IF(G20&lt;=E20,"Met","Not Met"),IF(F20="=",IF(G20=E20,"Met","Not Met"),""))))</f>

</xml_diff>